<commit_message>
fix: V7 Sheet2恢复类别展示区 + 修正MEMORY.md的API type映射
</commit_message>
<xml_diff>
--- a/config/成衣工艺单_设计师填表模板_v7.xlsx
+++ b/config/成衣工艺单_设计师填表模板_v7.xlsx
@@ -230,7 +230,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill/>
     </fill>
@@ -472,6 +472,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00595959"/>
       </patternFill>
     </fill>
   </fills>
@@ -794,7 +799,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -861,12 +866,18 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="42" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="40" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="40" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="41" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2190,15 +2201,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2226,12 +2246,12 @@
       </c>
       <c r="B2" s="26" t="inlineStr">
         <is>
+          <t>0.2边线</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
           <t>丝印烫标</t>
-        </is>
-      </c>
-      <c r="C2" s="26" t="inlineStr">
-        <is>
-          <t>0.2边线</t>
         </is>
       </c>
     </row>
@@ -2243,12 +2263,12 @@
       </c>
       <c r="B3" s="26" t="inlineStr">
         <is>
+          <t>0.5单线</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
           <t>吊染</t>
-        </is>
-      </c>
-      <c r="C3" s="26" t="inlineStr">
-        <is>
-          <t>0.5单线</t>
         </is>
       </c>
     </row>
@@ -2260,12 +2280,12 @@
       </c>
       <c r="B4" s="26" t="inlineStr">
         <is>
+          <t>2号反底</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
           <t>喷色</t>
-        </is>
-      </c>
-      <c r="C4" s="26" t="inlineStr">
-        <is>
-          <t>2号反底</t>
         </is>
       </c>
     </row>
@@ -2277,12 +2297,12 @@
       </c>
       <c r="B5" s="26" t="inlineStr">
         <is>
+          <t>三针五线大哈苏</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
           <t>喷马骝</t>
-        </is>
-      </c>
-      <c r="C5" s="26" t="inlineStr">
-        <is>
-          <t>三针五线大哈苏</t>
         </is>
       </c>
     </row>
@@ -2294,12 +2314,12 @@
       </c>
       <c r="B6" s="26" t="inlineStr">
         <is>
+          <t>三针四线</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
           <t>成衣刻字膜</t>
-        </is>
-      </c>
-      <c r="C6" s="26" t="inlineStr">
-        <is>
-          <t>三针四线</t>
         </is>
       </c>
     </row>
@@ -2311,12 +2331,12 @@
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
+          <t>两针四线大哈苏</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
           <t>手擦</t>
-        </is>
-      </c>
-      <c r="C7" s="26" t="inlineStr">
-        <is>
-          <t>两针四线大哈苏</t>
         </is>
       </c>
     </row>
@@ -2328,12 +2348,12 @@
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
+          <t>分中坎</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
           <t>扎染</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="inlineStr">
-        <is>
-          <t>分中坎</t>
         </is>
       </c>
     </row>
@@ -2345,12 +2365,12 @@
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
+          <t>压胶</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
           <t>无缝压胶</t>
-        </is>
-      </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>压胶</t>
         </is>
       </c>
     </row>
@@ -2362,12 +2382,12 @@
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
+          <t>哨牙线</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
           <t>普洗</t>
-        </is>
-      </c>
-      <c r="C10" s="26" t="inlineStr">
-        <is>
-          <t>哨牙线</t>
         </is>
       </c>
     </row>
@@ -2379,12 +2399,12 @@
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
+          <t>坎双线</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
           <t>水床冲孔</t>
-        </is>
-      </c>
-      <c r="C11" s="26" t="inlineStr">
-        <is>
-          <t>坎双线</t>
         </is>
       </c>
     </row>
@@ -2396,12 +2416,12 @@
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
+          <t>小两针四线小哈苏</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
           <t>激光烧花</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="inlineStr">
-        <is>
-          <t>小两针四线小哈苏</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2433,12 @@
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
+          <t>小分中坎</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
           <t>炒盐</t>
-        </is>
-      </c>
-      <c r="C13" s="26" t="inlineStr">
-        <is>
-          <t>小分中坎</t>
         </is>
       </c>
     </row>
@@ -2430,12 +2450,12 @@
       </c>
       <c r="B14" s="26" t="inlineStr">
         <is>
+          <t>小双线（窄针）</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
           <t>炒色</t>
-        </is>
-      </c>
-      <c r="C14" s="26" t="inlineStr">
-        <is>
-          <t>小双线（窄针）</t>
         </is>
       </c>
     </row>
@@ -2447,12 +2467,12 @@
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
+          <t>峰哥工艺线（高弹丝）</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
           <t>炒雪花</t>
-        </is>
-      </c>
-      <c r="C15" s="26" t="inlineStr">
-        <is>
-          <t>峰哥工艺线（高弹丝）</t>
         </is>
       </c>
     </row>
@@ -2464,12 +2484,12 @@
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
+          <t>来去缝</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
           <t>砂洗</t>
-        </is>
-      </c>
-      <c r="C16" s="26" t="inlineStr">
-        <is>
-          <t>来去缝</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2501,12 @@
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
+          <t>牙签线</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
           <t>破坏</t>
-        </is>
-      </c>
-      <c r="C17" s="26" t="inlineStr">
-        <is>
-          <t>牙签线</t>
         </is>
       </c>
     </row>
@@ -2498,12 +2518,12 @@
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
+          <t>落行窄针小双线</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
           <t>背胶章仔绣</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="inlineStr">
-        <is>
-          <t>落行窄针小双线</t>
         </is>
       </c>
     </row>
@@ -2515,12 +2535,12 @@
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
+          <t>龅牙线</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
           <t>酵洗</t>
-        </is>
-      </c>
-      <c r="C19" s="26" t="inlineStr">
-        <is>
-          <t>龅牙线</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2550,7 @@
           <t>吊染</t>
         </is>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>高弹肤感硅胶</t>
         </is>
@@ -2872,325 +2892,310 @@
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="27" t="inlineStr">
-        <is>
-          <t>工艺制作（类别展示）</t>
-        </is>
-      </c>
-    </row>
     <row r="72">
-      <c r="A72" s="28" t="inlineStr">
+      <c r="A72" s="27" t="inlineStr">
+        <is>
+          <t>工艺制作（类别展示，仅供设计师参考）</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="28" t="inlineStr">
         <is>
           <t>洗水</t>
         </is>
       </c>
-      <c r="B72" s="28" t="inlineStr">
+      <c r="B73" s="28" t="inlineStr">
         <is>
           <t>热转压印</t>
         </is>
       </c>
-      <c r="C72" s="28" t="inlineStr">
+      <c r="C73" s="28" t="inlineStr">
         <is>
           <t>直喷印花</t>
         </is>
       </c>
-      <c r="D72" s="28" t="inlineStr">
+      <c r="D73" s="28" t="inlineStr">
         <is>
           <t>绣花</t>
         </is>
       </c>
-      <c r="E72" s="28" t="inlineStr">
+      <c r="E73" s="28" t="inlineStr">
         <is>
           <t>网板印花</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="29" t="inlineStr">
-        <is>
-          <t>吊染</t>
-        </is>
-      </c>
-      <c r="B73" s="29" t="inlineStr">
-        <is>
-          <t>丝印刻字膜烫标</t>
-        </is>
-      </c>
-      <c r="C73" s="29" t="inlineStr">
-        <is>
-          <t>数码直喷/不打底</t>
-        </is>
-      </c>
-      <c r="D73" s="29" t="inlineStr">
-        <is>
-          <t>V字针绣</t>
-        </is>
-      </c>
-      <c r="E73" s="29" t="inlineStr">
-        <is>
-          <t>仿拨印</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="29" t="inlineStr">
         <is>
-          <t>喷色</t>
+          <t>吊染</t>
         </is>
       </c>
       <c r="B74" s="29" t="inlineStr">
         <is>
-          <t>丝印烫标（加防升华）</t>
+          <t>丝印刻字膜烫标</t>
         </is>
       </c>
       <c r="C74" s="29" t="inlineStr">
         <is>
-          <t>数码直喷/打底</t>
+          <t>数码直喷/不打底</t>
         </is>
       </c>
       <c r="D74" s="29" t="inlineStr">
         <is>
-          <t>一字绣（特种专机）</t>
+          <t>V字针绣</t>
         </is>
       </c>
       <c r="E74" s="29" t="inlineStr">
         <is>
-          <t>光感印</t>
+          <t>仿拨印</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="29" t="inlineStr">
         <is>
-          <t>喷马骝</t>
+          <t>喷色</t>
         </is>
       </c>
       <c r="B75" s="29" t="inlineStr">
         <is>
-          <t>刻字膜</t>
+          <t>丝印烫标（加防升华）</t>
         </is>
       </c>
       <c r="C75" s="29" t="inlineStr">
         <is>
-          <t>热转印/热升华</t>
+          <t>数码直喷/打底</t>
         </is>
       </c>
       <c r="D75" s="29" t="inlineStr">
         <is>
-          <t>中空绣</t>
+          <t>一字绣（特种专机）</t>
         </is>
       </c>
       <c r="E75" s="29" t="inlineStr">
         <is>
-          <t>厚板印</t>
+          <t>光感印</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="29" t="inlineStr">
         <is>
-          <t>手擦</t>
+          <t>喷马骝</t>
         </is>
       </c>
       <c r="B76" s="29" t="inlineStr">
         <is>
-          <t>压褶</t>
+          <t>刻字膜</t>
         </is>
       </c>
       <c r="C76" s="29" t="inlineStr">
         <is>
-          <t>白墨直喷/不打底</t>
+          <t>热转印/热升华</t>
         </is>
       </c>
       <c r="D76" s="29" t="inlineStr">
         <is>
-          <t>人字车</t>
+          <t>中空绣</t>
         </is>
       </c>
       <c r="E76" s="29" t="inlineStr">
         <is>
-          <t>反光浆</t>
+          <t>厚板印</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="29" t="inlineStr">
         <is>
-          <t>扎染</t>
+          <t>手擦</t>
         </is>
       </c>
       <c r="B77" s="29" t="inlineStr">
         <is>
-          <t>厚版肤感弹力硅胶章</t>
+          <t>压褶</t>
         </is>
       </c>
       <c r="C77" s="29" t="inlineStr">
         <is>
-          <t>白墨直喷/打底</t>
+          <t>白墨直喷/不打底</t>
         </is>
       </c>
       <c r="D77" s="29" t="inlineStr">
         <is>
-          <t>充棉工艺</t>
+          <t>人字车</t>
         </is>
       </c>
       <c r="E77" s="29" t="inlineStr">
         <is>
-          <t>发泡印</t>
+          <t>反光浆</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="29" t="inlineStr">
         <is>
-          <t>炒盐</t>
+          <t>扎染</t>
         </is>
       </c>
       <c r="B78" s="29" t="inlineStr">
         <is>
-          <t>反光刻字膜</t>
-        </is>
-      </c>
-      <c r="C78" s="29" t="inlineStr"/>
+          <t>厚版肤感弹力硅胶章</t>
+        </is>
+      </c>
+      <c r="C78" s="29" t="inlineStr">
+        <is>
+          <t>白墨直喷/打底</t>
+        </is>
+      </c>
       <c r="D78" s="29" t="inlineStr">
         <is>
-          <t>包边绣</t>
+          <t>充棉工艺</t>
         </is>
       </c>
       <c r="E78" s="29" t="inlineStr">
         <is>
-          <t>哑光胶浆</t>
+          <t>发泡印</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="29" t="inlineStr">
         <is>
-          <t>炒色</t>
+          <t>炒盐</t>
         </is>
       </c>
       <c r="B79" s="29" t="inlineStr">
         <is>
-          <t>激光冲孔</t>
+          <t>反光刻字膜</t>
         </is>
       </c>
       <c r="C79" s="29" t="inlineStr"/>
       <c r="D79" s="29" t="inlineStr">
         <is>
-          <t>十字绣</t>
+          <t>包边绣</t>
         </is>
       </c>
       <c r="E79" s="29" t="inlineStr">
         <is>
-          <t>彩色硅胶印</t>
+          <t>哑光胶浆</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="29" t="inlineStr">
         <is>
-          <t>炒雪花</t>
+          <t>炒色</t>
         </is>
       </c>
       <c r="B80" s="29" t="inlineStr">
         <is>
-          <t>烫画</t>
+          <t>激光冲孔</t>
         </is>
       </c>
       <c r="C80" s="29" t="inlineStr"/>
       <c r="D80" s="29" t="inlineStr">
         <is>
-          <t>平绣</t>
+          <t>十字绣</t>
         </is>
       </c>
       <c r="E80" s="29" t="inlineStr">
         <is>
-          <t>拉浆/石头浆</t>
+          <t>彩色硅胶印</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="29" t="inlineStr">
         <is>
-          <t>砂洗</t>
+          <t>炒雪花</t>
         </is>
       </c>
       <c r="B81" s="29" t="inlineStr">
         <is>
-          <t>热转印</t>
+          <t>烫画</t>
         </is>
       </c>
       <c r="C81" s="29" t="inlineStr"/>
       <c r="D81" s="29" t="inlineStr">
         <is>
-          <t>挨针绣</t>
+          <t>平绣</t>
         </is>
       </c>
       <c r="E81" s="29" t="inlineStr">
         <is>
-          <t>拨印</t>
+          <t>拉浆/石头浆</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="29" t="inlineStr">
         <is>
-          <t>碧纹染</t>
+          <t>砂洗</t>
         </is>
       </c>
       <c r="B82" s="29" t="inlineStr">
         <is>
-          <t>立体钢印</t>
+          <t>热转印</t>
         </is>
       </c>
       <c r="C82" s="29" t="inlineStr"/>
       <c r="D82" s="29" t="inlineStr">
         <is>
-          <t>明星特种专机-207</t>
+          <t>挨针绣</t>
         </is>
       </c>
       <c r="E82" s="29" t="inlineStr">
         <is>
-          <t>植绒印花</t>
+          <t>拨印</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="29" t="inlineStr">
         <is>
-          <t>酵洗</t>
+          <t>碧纹染</t>
         </is>
       </c>
       <c r="B83" s="29" t="inlineStr">
         <is>
-          <t>高周波</t>
+          <t>立体钢印</t>
         </is>
       </c>
       <c r="C83" s="29" t="inlineStr"/>
       <c r="D83" s="29" t="inlineStr">
         <is>
-          <t>榻榻米绣</t>
+          <t>明星特种专机-207</t>
         </is>
       </c>
       <c r="E83" s="29" t="inlineStr">
         <is>
-          <t>水显印</t>
+          <t>植绒印花</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="29" t="inlineStr"/>
-      <c r="B84" s="29" t="inlineStr"/>
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>酵洗</t>
+        </is>
+      </c>
+      <c r="B84" s="29" t="inlineStr">
+        <is>
+          <t>高周波</t>
+        </is>
+      </c>
       <c r="C84" s="29" t="inlineStr"/>
       <c r="D84" s="29" t="inlineStr">
         <is>
-          <t>毛巾绣</t>
+          <t>榻榻米绣</t>
         </is>
       </c>
       <c r="E84" s="29" t="inlineStr">
         <is>
-          <t>水浆</t>
+          <t>水显印</t>
         </is>
       </c>
     </row>
@@ -3200,12 +3205,12 @@
       <c r="C85" s="29" t="inlineStr"/>
       <c r="D85" s="29" t="inlineStr">
         <is>
-          <t>牙刷绣</t>
+          <t>毛巾绣</t>
         </is>
       </c>
       <c r="E85" s="29" t="inlineStr">
         <is>
-          <t>活性印花</t>
+          <t>水浆</t>
         </is>
       </c>
     </row>
@@ -3215,12 +3220,12 @@
       <c r="C86" s="29" t="inlineStr"/>
       <c r="D86" s="29" t="inlineStr">
         <is>
-          <t>珠片绣</t>
+          <t>牙刷绣</t>
         </is>
       </c>
       <c r="E86" s="29" t="inlineStr">
         <is>
-          <t>温变印</t>
+          <t>活性印花</t>
         </is>
       </c>
     </row>
@@ -3230,12 +3235,12 @@
       <c r="C87" s="29" t="inlineStr"/>
       <c r="D87" s="29" t="inlineStr">
         <is>
-          <t>立体绣</t>
+          <t>珠片绣</t>
         </is>
       </c>
       <c r="E87" s="29" t="inlineStr">
         <is>
-          <t>烫金/烫银</t>
+          <t>温变印</t>
         </is>
       </c>
     </row>
@@ -3245,12 +3250,12 @@
       <c r="C88" s="29" t="inlineStr"/>
       <c r="D88" s="29" t="inlineStr">
         <is>
-          <t>绳绣</t>
+          <t>立体绣</t>
         </is>
       </c>
       <c r="E88" s="29" t="inlineStr">
         <is>
-          <t>热固油墨</t>
+          <t>烫金/烫银</t>
         </is>
       </c>
     </row>
@@ -3260,12 +3265,12 @@
       <c r="C89" s="29" t="inlineStr"/>
       <c r="D89" s="29" t="inlineStr">
         <is>
-          <t>菱形打边绣（特种专机）</t>
+          <t>绳绣</t>
         </is>
       </c>
       <c r="E89" s="29" t="inlineStr">
         <is>
-          <t>硅胶印</t>
+          <t>热固油墨</t>
         </is>
       </c>
     </row>
@@ -3275,12 +3280,12 @@
       <c r="C90" s="29" t="inlineStr"/>
       <c r="D90" s="29" t="inlineStr">
         <is>
-          <t>贴布绣</t>
+          <t>菱形打边绣（特种专机）</t>
         </is>
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>网点印</t>
+          <t>硅胶印</t>
         </is>
       </c>
     </row>
@@ -3290,12 +3295,12 @@
       <c r="C91" s="29" t="inlineStr"/>
       <c r="D91" s="29" t="inlineStr">
         <is>
-          <t>锁链绣</t>
+          <t>贴布绣</t>
         </is>
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>裂纹印</t>
+          <t>网点印</t>
         </is>
       </c>
     </row>
@@ -3305,227 +3310,383 @@
       <c r="C92" s="29" t="inlineStr"/>
       <c r="D92" s="29" t="inlineStr">
         <is>
+          <t>锁链绣</t>
+        </is>
+      </c>
+      <c r="E92" s="29" t="inlineStr">
+        <is>
+          <t>裂纹印</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="29" t="inlineStr"/>
+      <c r="B93" s="29" t="inlineStr"/>
+      <c r="C93" s="29" t="inlineStr"/>
+      <c r="D93" s="29" t="inlineStr">
+        <is>
           <t>镂空绣</t>
         </is>
       </c>
-      <c r="E92" s="29" t="inlineStr">
+      <c r="E93" s="29" t="inlineStr">
         <is>
           <t>轻薄热固油墨</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="27" t="inlineStr">
-        <is>
-          <t>车缝工艺（类别展示）</t>
-        </is>
-      </c>
-    </row>
     <row r="96">
-      <c r="A96" s="28" t="inlineStr">
+      <c r="A96" s="30" t="inlineStr">
+        <is>
+          <t>车缝工艺（类别展示，仅供设计师参考）</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="28" t="inlineStr">
+        <is>
+          <t>车缝工艺</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="29" t="inlineStr">
+        <is>
+          <t>0.2边线</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="29" t="inlineStr">
+        <is>
+          <t>0.5单线</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="29" t="inlineStr">
+        <is>
+          <t>2号反底</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="29" t="inlineStr">
+        <is>
+          <t>三针五线大哈苏</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="29" t="inlineStr">
+        <is>
+          <t>三针四线</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="29" t="inlineStr">
+        <is>
+          <t>两针四线大哈苏</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="29" t="inlineStr">
+        <is>
+          <t>分中坎</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="29" t="inlineStr">
+        <is>
+          <t>压胶</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="29" t="inlineStr">
+        <is>
+          <t>哨牙线</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="29" t="inlineStr">
+        <is>
+          <t>坎双线</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="29" t="inlineStr">
+        <is>
+          <t>小两针四线小哈苏</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="29" t="inlineStr">
+        <is>
+          <t>小分中坎</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="29" t="inlineStr">
+        <is>
+          <t>小双线（窄针）</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="29" t="inlineStr">
+        <is>
+          <t>峰哥工艺线（高弹丝）</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="29" t="inlineStr">
+        <is>
+          <t>来去缝</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="29" t="inlineStr">
+        <is>
+          <t>牙签线</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="29" t="inlineStr">
+        <is>
+          <t>落行窄针小双线</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="29" t="inlineStr">
+        <is>
+          <t>龅牙线</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="31" t="inlineStr">
+        <is>
+          <t>成衣工艺（类别展示，仅供设计师参考）</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="28" t="inlineStr">
         <is>
           <t>无缝</t>
         </is>
       </c>
-      <c r="B96" s="28" t="inlineStr">
+      <c r="B119" s="28" t="inlineStr">
         <is>
           <t>洗水</t>
         </is>
       </c>
-      <c r="C96" s="28" t="inlineStr">
+      <c r="C119" s="28" t="inlineStr">
         <is>
           <t>热转压印</t>
         </is>
       </c>
-      <c r="D96" s="28" t="inlineStr">
+      <c r="D119" s="28" t="inlineStr">
         <is>
           <t>绣花</t>
         </is>
       </c>
-      <c r="E96" s="28" t="inlineStr">
+      <c r="E119" s="28" t="inlineStr">
         <is>
           <t>网板印花</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="29" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="29" t="inlineStr">
         <is>
           <t>无缝压胶</t>
         </is>
       </c>
-      <c r="B97" s="29" t="inlineStr">
+      <c r="B120" s="29" t="inlineStr">
         <is>
           <t>吊染</t>
         </is>
       </c>
-      <c r="C97" s="29" t="inlineStr">
+      <c r="C120" s="29" t="inlineStr">
         <is>
           <t>成衣刻字膜</t>
         </is>
       </c>
-      <c r="D97" s="29" t="inlineStr">
+      <c r="D120" s="29" t="inlineStr">
         <is>
           <t>背胶章仔绣</t>
         </is>
       </c>
-      <c r="E97" s="29" t="inlineStr">
+      <c r="E120" s="29" t="inlineStr">
         <is>
           <t>丝印烫标</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="29" t="inlineStr"/>
-      <c r="B98" s="29" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="29" t="inlineStr"/>
+      <c r="B121" s="29" t="inlineStr">
         <is>
           <t>喷色</t>
         </is>
       </c>
-      <c r="C98" s="29" t="inlineStr">
+      <c r="C121" s="29" t="inlineStr">
         <is>
           <t>高弹肤感硅胶</t>
         </is>
       </c>
-      <c r="D98" s="29" t="inlineStr"/>
-      <c r="E98" s="29" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="29" t="inlineStr"/>
-      <c r="B99" s="29" t="inlineStr">
+      <c r="D121" s="29" t="inlineStr"/>
+      <c r="E121" s="29" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="29" t="inlineStr"/>
+      <c r="B122" s="29" t="inlineStr">
         <is>
           <t>喷马骝</t>
         </is>
       </c>
-      <c r="C99" s="29" t="inlineStr"/>
-      <c r="D99" s="29" t="inlineStr"/>
-      <c r="E99" s="29" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="29" t="inlineStr"/>
-      <c r="B100" s="29" t="inlineStr">
+      <c r="C122" s="29" t="inlineStr"/>
+      <c r="D122" s="29" t="inlineStr"/>
+      <c r="E122" s="29" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="29" t="inlineStr"/>
+      <c r="B123" s="29" t="inlineStr">
         <is>
           <t>手擦</t>
         </is>
       </c>
-      <c r="C100" s="29" t="inlineStr"/>
-      <c r="D100" s="29" t="inlineStr"/>
-      <c r="E100" s="29" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="29" t="inlineStr"/>
-      <c r="B101" s="29" t="inlineStr">
+      <c r="C123" s="29" t="inlineStr"/>
+      <c r="D123" s="29" t="inlineStr"/>
+      <c r="E123" s="29" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="29" t="inlineStr"/>
+      <c r="B124" s="29" t="inlineStr">
         <is>
           <t>扎染</t>
         </is>
       </c>
-      <c r="C101" s="29" t="inlineStr"/>
-      <c r="D101" s="29" t="inlineStr"/>
-      <c r="E101" s="29" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="29" t="inlineStr"/>
-      <c r="B102" s="29" t="inlineStr">
+      <c r="C124" s="29" t="inlineStr"/>
+      <c r="D124" s="29" t="inlineStr"/>
+      <c r="E124" s="29" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="29" t="inlineStr"/>
+      <c r="B125" s="29" t="inlineStr">
         <is>
           <t>普洗</t>
         </is>
       </c>
-      <c r="C102" s="29" t="inlineStr"/>
-      <c r="D102" s="29" t="inlineStr"/>
-      <c r="E102" s="29" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="29" t="inlineStr"/>
-      <c r="B103" s="29" t="inlineStr">
+      <c r="C125" s="29" t="inlineStr"/>
+      <c r="D125" s="29" t="inlineStr"/>
+      <c r="E125" s="29" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="29" t="inlineStr"/>
+      <c r="B126" s="29" t="inlineStr">
         <is>
           <t>水床冲孔</t>
         </is>
       </c>
-      <c r="C103" s="29" t="inlineStr"/>
-      <c r="D103" s="29" t="inlineStr"/>
-      <c r="E103" s="29" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="29" t="inlineStr"/>
-      <c r="B104" s="29" t="inlineStr">
+      <c r="C126" s="29" t="inlineStr"/>
+      <c r="D126" s="29" t="inlineStr"/>
+      <c r="E126" s="29" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="29" t="inlineStr"/>
+      <c r="B127" s="29" t="inlineStr">
         <is>
           <t>激光烧花</t>
         </is>
       </c>
-      <c r="C104" s="29" t="inlineStr"/>
-      <c r="D104" s="29" t="inlineStr"/>
-      <c r="E104" s="29" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="29" t="inlineStr"/>
-      <c r="B105" s="29" t="inlineStr">
+      <c r="C127" s="29" t="inlineStr"/>
+      <c r="D127" s="29" t="inlineStr"/>
+      <c r="E127" s="29" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="29" t="inlineStr"/>
+      <c r="B128" s="29" t="inlineStr">
         <is>
           <t>炒盐</t>
         </is>
       </c>
-      <c r="C105" s="29" t="inlineStr"/>
-      <c r="D105" s="29" t="inlineStr"/>
-      <c r="E105" s="29" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="29" t="inlineStr"/>
-      <c r="B106" s="29" t="inlineStr">
+      <c r="C128" s="29" t="inlineStr"/>
+      <c r="D128" s="29" t="inlineStr"/>
+      <c r="E128" s="29" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="29" t="inlineStr"/>
+      <c r="B129" s="29" t="inlineStr">
         <is>
           <t>炒色</t>
         </is>
       </c>
-      <c r="C106" s="29" t="inlineStr"/>
-      <c r="D106" s="29" t="inlineStr"/>
-      <c r="E106" s="29" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="29" t="inlineStr"/>
-      <c r="B107" s="29" t="inlineStr">
+      <c r="C129" s="29" t="inlineStr"/>
+      <c r="D129" s="29" t="inlineStr"/>
+      <c r="E129" s="29" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="29" t="inlineStr"/>
+      <c r="B130" s="29" t="inlineStr">
         <is>
           <t>炒雪花</t>
         </is>
       </c>
-      <c r="C107" s="29" t="inlineStr"/>
-      <c r="D107" s="29" t="inlineStr"/>
-      <c r="E107" s="29" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="29" t="inlineStr"/>
-      <c r="B108" s="29" t="inlineStr">
+      <c r="C130" s="29" t="inlineStr"/>
+      <c r="D130" s="29" t="inlineStr"/>
+      <c r="E130" s="29" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="29" t="inlineStr"/>
+      <c r="B131" s="29" t="inlineStr">
         <is>
           <t>砂洗</t>
         </is>
       </c>
-      <c r="C108" s="29" t="inlineStr"/>
-      <c r="D108" s="29" t="inlineStr"/>
-      <c r="E108" s="29" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="29" t="inlineStr"/>
-      <c r="B109" s="29" t="inlineStr">
+      <c r="C131" s="29" t="inlineStr"/>
+      <c r="D131" s="29" t="inlineStr"/>
+      <c r="E131" s="29" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="29" t="inlineStr"/>
+      <c r="B132" s="29" t="inlineStr">
         <is>
           <t>破坏</t>
         </is>
       </c>
-      <c r="C109" s="29" t="inlineStr"/>
-      <c r="D109" s="29" t="inlineStr"/>
-      <c r="E109" s="29" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="29" t="inlineStr"/>
-      <c r="B110" s="29" t="inlineStr">
+      <c r="C132" s="29" t="inlineStr"/>
+      <c r="D132" s="29" t="inlineStr"/>
+      <c r="E132" s="29" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="29" t="inlineStr"/>
+      <c r="B133" s="29" t="inlineStr">
         <is>
           <t>酵洗</t>
         </is>
       </c>
-      <c r="C110" s="29" t="inlineStr"/>
-      <c r="D110" s="29" t="inlineStr"/>
-      <c r="E110" s="29" t="inlineStr"/>
+      <c r="C133" s="29" t="inlineStr"/>
+      <c r="D133" s="29" t="inlineStr"/>
+      <c r="E133" s="29" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A95:E95"/>
-    <mergeCell ref="A71:E71"/>
+  <mergeCells count="3">
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A96"/>
+    <mergeCell ref="A118:E118"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>